<commit_message>
Calibrated FG ageing: rebuild on live data incl. the 29-Oct invoices
Hyderabad (JODLTE1026/02054, 28.27 MT) and Tapi (JODLGJ1026/02488, 25.18 MT)
invoices dated 29-Oct arrived in the 12:36 UTC upload during verification.
System FG: Hyderabad 655.155, Tapi 759.585; calibrated totals unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SVVKmwQKKV189dev92iFna
</commit_message>
<xml_diff>
--- a/reports/FG-Ageing-Calibrated-2026-10-29.xlsx
+++ b/reports/FG-Ageing-Calibrated-2026-10-29.xlsx
@@ -119,7 +119,7 @@
     <t xml:space="preserve">FG ageing calibrated to plant FG sheets - by plant and size (29-Oct-2026)</t>
   </si>
   <si>
-    <t xml:space="preserve">System FG and FIFO ageing from the database (production to 28-Oct, invoices to 24-28 Oct by plant). Thickness clubbed to 1.6 / 2 / 2.5 / 3 / 4 / 5 / 6. Each size is calibrated to the plant sheet: ratio = plant FG / system FG, and every age bucket is multiplied by it. Plant stock the system shows as nil is "Age unknown".</t>
+    <t xml:space="preserve">System FG and FIFO ageing from the database (production to 26-28 Oct and invoices to 24-29 Oct, by plant). Thickness clubbed to 1.6 / 2 / 2.5 / 3 / 4 / 5 / 6. Each size is calibrated to the plant sheet: ratio = plant FG / system FG, and every age bucket is multiplied by it. Plant stock the system shows as nil is "Age unknown".</t>
   </si>
   <si>
     <t xml:space="preserve">Size</t>
@@ -1248,7 +1248,7 @@
       </c>
       <c r="B4" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$A$5:$A$171,A4,'Plant x size'!$C$5:$C$171)</f>
-        <v>683.42496592272</v>
+        <v>655.15496592272</v>
       </c>
       <c r="C4" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$A$5:$A$171,A4,'Plant x size'!$D$5:$D$171)</f>
@@ -1256,15 +1256,15 @@
       </c>
       <c r="D4" s="9" t="n">
         <f aca="false">IF(B4&gt;0,C4/B4,0)</f>
-        <v>0.941481555522744</v>
+        <v>0.982106575493618</v>
       </c>
       <c r="E4" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$A$5:$A$171,A4,'Plant x size'!$K$5:$K$171)</f>
-        <v>325.276515398259</v>
+        <v>326.85578916002</v>
       </c>
       <c r="F4" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$A$5:$A$171,A4,'Plant x size'!$L$5:$L$171)</f>
-        <v>89.235476583338</v>
+        <v>87.6562028215772</v>
       </c>
       <c r="G4" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$A$5:$A$171,A4,'Plant x size'!$M$5:$M$171)</f>
@@ -1292,7 +1292,7 @@
       </c>
       <c r="M4" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$A$5:$A$171,A4,'Plant x size'!$I$5:$I$171)+SUMIF('Plant x size'!$A$5:$A$171,A4,'Plant x size'!$J$5:$J$171)</f>
-        <v>241.077166636955</v>
+        <v>239.037166636955</v>
       </c>
       <c r="N4" s="8" t="n">
         <v>649.586</v>
@@ -1416,7 +1416,7 @@
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$A$5:$A$171,A7,'Plant x size'!$C$5:$C$171)</f>
-        <v>784.7645037</v>
+        <v>759.5845037</v>
       </c>
       <c r="C7" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$A$5:$A$171,A7,'Plant x size'!$D$5:$D$171)</f>
@@ -1424,15 +1424,15 @@
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">IF(B7&gt;0,C7/B7,0)</f>
-        <v>1.05381932554399</v>
+        <v>1.08875312222882</v>
       </c>
       <c r="E7" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$A$5:$A$171,A7,'Plant x size'!$K$5:$K$171)</f>
-        <v>731.339950729971</v>
+        <v>731.365841853333</v>
       </c>
       <c r="F7" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$A$5:$A$171,A7,'Plant x size'!$L$5:$L$171)</f>
-        <v>24.6600492700294</v>
+        <v>24.6341581466672</v>
       </c>
       <c r="G7" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$A$5:$A$171,A7,'Plant x size'!$M$5:$M$171)</f>
@@ -1472,7 +1472,7 @@
       </c>
       <c r="B8" s="12" t="n">
         <f aca="false">SUM(B4:B7)</f>
-        <v>2573.49662731872</v>
+        <v>2520.04662731872</v>
       </c>
       <c r="C8" s="12" t="n">
         <f aca="false">SUM(C4:C7)</f>
@@ -1480,15 +1480,15 @@
       </c>
       <c r="D8" s="13" t="n">
         <f aca="false">IF(B8&gt;0,C8/B8,0)</f>
-        <v>1.02224031384914</v>
+        <v>1.0439219542533</v>
       </c>
       <c r="E8" s="12" t="n">
         <f aca="false">SUM(E4:E7)</f>
-        <v>1997.16039909105</v>
+        <v>1998.76556397618</v>
       </c>
       <c r="F8" s="12" t="n">
         <f aca="false">SUM(F4:F7)</f>
-        <v>315.051592890545</v>
+        <v>313.446428005422</v>
       </c>
       <c r="G8" s="12" t="n">
         <f aca="false">SUM(G4:G7)</f>
@@ -1516,7 +1516,7 @@
       </c>
       <c r="M8" s="12" t="n">
         <f aca="false">SUM(M4:M7)</f>
-        <v>245.571414636955</v>
+        <v>243.531414636955</v>
       </c>
       <c r="N8" s="12" t="n">
         <f aca="false">SUM(N4:N7)</f>
@@ -1680,21 +1680,21 @@
         <v>42</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>12.3127576</v>
+        <v>8.21275760000001</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>11.749</v>
       </c>
       <c r="E5" s="20" t="n">
         <f aca="false">IF(C5&gt;0,D5/C5,"")</f>
-        <v>0.954213538647101</v>
+        <v>1.43057917598834</v>
       </c>
       <c r="F5" s="18" t="str">
         <f aca="false">IF(AND(C5=0,D5&gt;0),"Plant only",IF(AND(D5=0,C5&gt;0),"System only",IF(ABS(D5-C5)&lt;=0.5,"Match",IF(D5&gt;C5,"Plant more","Plant less"))))</f>
-        <v>Plant less</v>
+        <v>Plant more</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>12.3127576</v>
+        <v>8.21275760000001</v>
       </c>
       <c r="H5" s="8" t="n">
         <v>0</v>
@@ -1734,10 +1734,10 @@
         <v>0</v>
       </c>
       <c r="R5" s="21" t="n">
-        <v>11.4840348030566</v>
+        <v>9</v>
       </c>
       <c r="S5" s="22" t="n">
-        <v>28</v>
+        <v>9</v>
       </c>
       <c r="T5" s="23" t="n">
         <v>46315</v>
@@ -3163,21 +3163,21 @@
         <v>63</v>
       </c>
       <c r="C26" s="8" t="n">
-        <v>11.3509284</v>
+        <v>7.2709284</v>
       </c>
       <c r="D26" s="8" t="n">
         <v>16.866</v>
       </c>
       <c r="E26" s="20" t="n">
         <f aca="false">IF(C26&gt;0,D26/C26,"")</f>
-        <v>1.48586964921742</v>
+        <v>2.31964875352094</v>
       </c>
       <c r="F26" s="18" t="str">
         <f aca="false">IF(AND(C26=0,D26&gt;0),"Plant only",IF(AND(D26=0,C26&gt;0),"System only",IF(ABS(D26-C26)&lt;=0.5,"Match",IF(D26&gt;C26,"Plant more","Plant less"))))</f>
         <v>Plant more</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>11.3509284</v>
+        <v>7.2709284</v>
       </c>
       <c r="H26" s="8" t="n">
         <v>0</v>
@@ -3447,21 +3447,21 @@
         <v>67</v>
       </c>
       <c r="C30" s="8" t="n">
-        <v>20.6869648</v>
+        <v>16.6869648</v>
       </c>
       <c r="D30" s="8" t="n">
         <v>22.891</v>
       </c>
       <c r="E30" s="20" t="n">
         <f aca="false">IF(C30&gt;0,D30/C30,"")</f>
-        <v>1.10654222218235</v>
+        <v>1.37178931425564</v>
       </c>
       <c r="F30" s="18" t="str">
         <f aca="false">IF(AND(C30=0,D30&gt;0),"Plant only",IF(AND(D30=0,C30&gt;0),"System only",IF(ABS(D30-C30)&lt;=0.5,"Match",IF(D30&gt;C30,"Plant more","Plant less"))))</f>
         <v>Plant more</v>
       </c>
       <c r="G30" s="8" t="n">
-        <v>20.6869648</v>
+        <v>16.6869648</v>
       </c>
       <c r="H30" s="8" t="n">
         <v>0</v>
@@ -3873,21 +3873,21 @@
         <v>73</v>
       </c>
       <c r="C36" s="8" t="n">
-        <v>35.7587936</v>
+        <v>29.7587936</v>
       </c>
       <c r="D36" s="8" t="n">
         <v>28.752</v>
       </c>
       <c r="E36" s="20" t="n">
         <f aca="false">IF(C36&gt;0,D36/C36,"")</f>
-        <v>0.804053971216748</v>
+        <v>0.966168198431271</v>
       </c>
       <c r="F36" s="18" t="str">
         <f aca="false">IF(AND(C36=0,D36&gt;0),"Plant only",IF(AND(D36=0,C36&gt;0),"System only",IF(ABS(D36-C36)&lt;=0.5,"Match",IF(D36&gt;C36,"Plant more","Plant less"))))</f>
         <v>Plant less</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>35.7587936</v>
+        <v>29.7587936</v>
       </c>
       <c r="H36" s="8" t="n">
         <v>0</v>
@@ -3944,14 +3944,14 @@
         <v>74</v>
       </c>
       <c r="C37" s="8" t="n">
-        <v>21.946045</v>
+        <v>20.046045</v>
       </c>
       <c r="D37" s="8" t="n">
         <v>18.884</v>
       </c>
       <c r="E37" s="20" t="n">
         <f aca="false">IF(C37&gt;0,D37/C37,"")</f>
-        <v>0.86047394872288</v>
+        <v>0.942031208649885</v>
       </c>
       <c r="F37" s="18" t="str">
         <f aca="false">IF(AND(C37=0,D37&gt;0),"Plant only",IF(AND(D37=0,C37&gt;0),"System only",IF(ABS(D37-C37)&lt;=0.5,"Match",IF(D37&gt;C37,"Plant more","Plant less"))))</f>
@@ -3961,7 +3961,7 @@
         <v>19.3639875</v>
       </c>
       <c r="H37" s="8" t="n">
-        <v>2.58205749999999</v>
+        <v>0.682057500000017</v>
       </c>
       <c r="I37" s="8" t="n">
         <v>0</v>
@@ -3971,11 +3971,11 @@
       </c>
       <c r="K37" s="8" t="n">
         <f aca="false">IF(C37&gt;0,G37*E37,0)</f>
-        <v>16.6622067871455</v>
+        <v>18.2414805489063</v>
       </c>
       <c r="L37" s="8" t="n">
         <f aca="false">IF(C37&gt;0,H37*E37,0)</f>
-        <v>2.22179321285452</v>
+        <v>0.642519451093735</v>
       </c>
       <c r="M37" s="8" t="n">
         <f aca="false">IF(C37&gt;0,I37*E37,0)</f>
@@ -3998,7 +3998,7 @@
         <v>0</v>
       </c>
       <c r="R37" s="21" t="n">
-        <v>8.77532500730769</v>
+        <v>5.15232194180951</v>
       </c>
       <c r="S37" s="22" t="n">
         <v>47</v>
@@ -4228,21 +4228,21 @@
         <v>78</v>
       </c>
       <c r="C41" s="8" t="n">
-        <v>12.3371932480001</v>
+        <v>6.18719324800005</v>
       </c>
       <c r="D41" s="8" t="n">
         <v>8.726</v>
       </c>
       <c r="E41" s="20" t="n">
         <f aca="false">IF(C41&gt;0,D41/C41,"")</f>
-        <v>0.707292155078672</v>
+        <v>1.41033254502283</v>
       </c>
       <c r="F41" s="18" t="str">
         <f aca="false">IF(AND(C41=0,D41&gt;0),"Plant only",IF(AND(D41=0,C41&gt;0),"System only",IF(ABS(D41-C41)&lt;=0.5,"Match",IF(D41&gt;C41,"Plant more","Plant less"))))</f>
-        <v>Plant less</v>
+        <v>Plant more</v>
       </c>
       <c r="G41" s="8" t="n">
-        <v>12.3371932480001</v>
+        <v>6.18719324800005</v>
       </c>
       <c r="H41" s="8" t="n">
         <v>0</v>
@@ -4796,18 +4796,18 @@
         <v>86</v>
       </c>
       <c r="C49" s="8" t="n">
-        <v>9.04905037447167</v>
+        <v>7.00905037447168</v>
       </c>
       <c r="D49" s="8" t="n">
         <v>6.762</v>
       </c>
       <c r="E49" s="20" t="n">
         <f aca="false">IF(C49&gt;0,D49/C49,"")</f>
-        <v>0.747260731255991</v>
+        <v>0.964752661020745</v>
       </c>
       <c r="F49" s="18" t="str">
         <f aca="false">IF(AND(C49=0,D49&gt;0),"Plant only",IF(AND(D49=0,C49&gt;0),"System only",IF(ABS(D49-C49)&lt;=0.5,"Match",IF(D49&gt;C49,"Plant more","Plant less"))))</f>
-        <v>Plant less</v>
+        <v>Match</v>
       </c>
       <c r="G49" s="8" t="n">
         <v>0</v>
@@ -4816,7 +4816,7 @@
         <v>0</v>
       </c>
       <c r="I49" s="8" t="n">
-        <v>9.04905037447167</v>
+        <v>7.00905037447168</v>
       </c>
       <c r="J49" s="8" t="n">
         <v>0</v>
@@ -10367,21 +10367,21 @@
         <v>57</v>
       </c>
       <c r="C128" s="8" t="n">
-        <v>31.229184</v>
+        <v>25.189184</v>
       </c>
       <c r="D128" s="8" t="n">
         <v>33</v>
       </c>
       <c r="E128" s="20" t="n">
         <f aca="false">IF(C128&gt;0,D128/C128,"")</f>
-        <v>1.056703883137</v>
+        <v>1.31008610679885</v>
       </c>
       <c r="F128" s="18" t="str">
         <f aca="false">IF(AND(C128=0,D128&gt;0),"Plant only",IF(AND(D128=0,C128&gt;0),"System only",IF(ABS(D128-C128)&lt;=0.5,"Match",IF(D128&gt;C128,"Plant more","Plant less"))))</f>
         <v>Plant more</v>
       </c>
       <c r="G128" s="8" t="n">
-        <v>31.229184</v>
+        <v>25.189184</v>
       </c>
       <c r="H128" s="8" t="n">
         <v>0</v>
@@ -10438,21 +10438,21 @@
         <v>141</v>
       </c>
       <c r="C129" s="8" t="n">
-        <v>23.10726</v>
+        <v>18.13226</v>
       </c>
       <c r="D129" s="8" t="n">
         <v>23</v>
       </c>
       <c r="E129" s="20" t="n">
         <f aca="false">IF(C129&gt;0,D129/C129,"")</f>
-        <v>0.995358168817939</v>
+        <v>1.26845743442902</v>
       </c>
       <c r="F129" s="18" t="str">
         <f aca="false">IF(AND(C129=0,D129&gt;0),"Plant only",IF(AND(D129=0,C129&gt;0),"System only",IF(ABS(D129-C129)&lt;=0.5,"Match",IF(D129&gt;C129,"Plant more","Plant less"))))</f>
-        <v>Match</v>
+        <v>Plant more</v>
       </c>
       <c r="G129" s="8" t="n">
-        <v>23.10726</v>
+        <v>18.13226</v>
       </c>
       <c r="H129" s="8" t="n">
         <v>0</v>
@@ -10492,7 +10492,7 @@
         <v>0</v>
       </c>
       <c r="R129" s="21" t="n">
-        <v>1.38116591928251</v>
+        <v>1.21137464386679</v>
       </c>
       <c r="S129" s="22" t="n">
         <v>2</v>
@@ -11132,21 +11132,21 @@
         <v>121</v>
       </c>
       <c r="C139" s="8" t="n">
-        <v>30.3663824</v>
+        <v>27.2463824</v>
       </c>
       <c r="D139" s="8" t="n">
         <v>35</v>
       </c>
       <c r="E139" s="20" t="n">
         <f aca="false">IF(C139&gt;0,D139/C139,"")</f>
-        <v>1.15259037243765</v>
+        <v>1.28457420461074</v>
       </c>
       <c r="F139" s="18" t="str">
         <f aca="false">IF(AND(C139=0,D139&gt;0),"Plant only",IF(AND(D139=0,C139&gt;0),"System only",IF(ABS(D139-C139)&lt;=0.5,"Match",IF(D139&gt;C139,"Plant more","Plant less"))))</f>
         <v>Plant more</v>
       </c>
       <c r="G139" s="8" t="n">
-        <v>30.3663824</v>
+        <v>27.2463824</v>
       </c>
       <c r="H139" s="8" t="n">
         <v>0</v>
@@ -11186,7 +11186,7 @@
         <v>0</v>
       </c>
       <c r="R139" s="21" t="n">
-        <v>3.36705611663508</v>
+        <v>2.72202424935502</v>
       </c>
       <c r="S139" s="22" t="n">
         <v>9</v>
@@ -11203,21 +11203,21 @@
         <v>122</v>
       </c>
       <c r="C140" s="8" t="n">
-        <v>6.94151360000002</v>
+        <v>4.94651360000001</v>
       </c>
       <c r="D140" s="8" t="n">
         <v>12</v>
       </c>
       <c r="E140" s="20" t="n">
         <f aca="false">IF(C140&gt;0,D140/C140,"")</f>
-        <v>1.72872959580458</v>
+        <v>2.4259510779471</v>
       </c>
       <c r="F140" s="18" t="str">
         <f aca="false">IF(AND(C140=0,D140&gt;0),"Plant only",IF(AND(D140=0,C140&gt;0),"System only",IF(ABS(D140-C140)&lt;=0.5,"Match",IF(D140&gt;C140,"Plant more","Plant less"))))</f>
         <v>Plant more</v>
       </c>
       <c r="G140" s="8" t="n">
-        <v>6.94151360000002</v>
+        <v>4.94651360000001</v>
       </c>
       <c r="H140" s="8" t="n">
         <v>0</v>
@@ -11274,24 +11274,24 @@
         <v>123</v>
       </c>
       <c r="C141" s="8" t="n">
-        <v>20.16135</v>
+        <v>14.98635</v>
       </c>
       <c r="D141" s="8" t="n">
         <v>20</v>
       </c>
       <c r="E141" s="20" t="n">
         <f aca="false">IF(C141&gt;0,D141/C141,"")</f>
-        <v>0.991997063688692</v>
+        <v>1.33454777180568</v>
       </c>
       <c r="F141" s="18" t="str">
         <f aca="false">IF(AND(C141=0,D141&gt;0),"Plant only",IF(AND(D141=0,C141&gt;0),"System only",IF(ABS(D141-C141)&lt;=0.5,"Match",IF(D141&gt;C141,"Plant more","Plant less"))))</f>
-        <v>Match</v>
+        <v>Plant more</v>
       </c>
       <c r="G141" s="8" t="n">
-        <v>20.13525</v>
+        <v>14.98635</v>
       </c>
       <c r="H141" s="8" t="n">
-        <v>0.026099999999996</v>
+        <v>0</v>
       </c>
       <c r="I141" s="8" t="n">
         <v>0</v>
@@ -11301,11 +11301,11 @@
       </c>
       <c r="K141" s="8" t="n">
         <f aca="false">IF(C141&gt;0,G141*E141,0)</f>
-        <v>19.9741088766377</v>
+        <v>20</v>
       </c>
       <c r="L141" s="8" t="n">
         <f aca="false">IF(C141&gt;0,H141*E141,0)</f>
-        <v>0.0258911233622709</v>
+        <v>0</v>
       </c>
       <c r="M141" s="8" t="n">
         <f aca="false">IF(C141&gt;0,I141*E141,0)</f>
@@ -11328,10 +11328,10 @@
         <v>0</v>
       </c>
       <c r="R141" s="21" t="n">
-        <v>3.07378970158247</v>
+        <v>3</v>
       </c>
       <c r="S141" s="22" t="n">
-        <v>60</v>
+        <v>3</v>
       </c>
       <c r="T141" s="23" t="n">
         <v>46321</v>
@@ -12903,21 +12903,21 @@
         <v>133</v>
       </c>
       <c r="C164" s="8" t="n">
-        <v>49.1075198</v>
+        <v>45.2325198</v>
       </c>
       <c r="D164" s="8" t="n">
         <v>21</v>
       </c>
       <c r="E164" s="20" t="n">
         <f aca="false">IF(C164&gt;0,D164/C164,"")</f>
-        <v>0.427633081155933</v>
+        <v>0.464267745702728</v>
       </c>
       <c r="F164" s="18" t="str">
         <f aca="false">IF(AND(C164=0,D164&gt;0),"Plant only",IF(AND(D164=0,C164&gt;0),"System only",IF(ABS(D164-C164)&lt;=0.5,"Match",IF(D164&gt;C164,"Plant more","Plant less"))))</f>
         <v>Plant less</v>
       </c>
       <c r="G164" s="8" t="n">
-        <v>49.1075198</v>
+        <v>45.2325198</v>
       </c>
       <c r="H164" s="8" t="n">
         <v>0</v>
@@ -12957,7 +12957,7 @@
         <v>0</v>
       </c>
       <c r="R164" s="21" t="n">
-        <v>22.7046102499357</v>
+        <v>22.6793046669932</v>
       </c>
       <c r="S164" s="22" t="n">
         <v>23</v>
@@ -13460,7 +13460,7 @@
       </c>
       <c r="C172" s="12" t="n">
         <f aca="false">SUBTOTAL(9,C5:C171)</f>
-        <v>2573.49662731872</v>
+        <v>2520.04662731872</v>
       </c>
       <c r="D172" s="12" t="n">
         <f aca="false">SUBTOTAL(9,D5:D171)</f>
@@ -13470,15 +13470,15 @@
       <c r="F172" s="11"/>
       <c r="G172" s="12" t="n">
         <f aca="false">SUBTOTAL(9,G5:G171)</f>
-        <v>2010.72710874166</v>
+        <v>1961.24320874166</v>
       </c>
       <c r="H172" s="12" t="n">
         <f aca="false">SUBTOTAL(9,H5:H171)</f>
-        <v>317.198103940105</v>
+        <v>315.272003940105</v>
       </c>
       <c r="I172" s="12" t="n">
         <f aca="false">SUBTOTAL(9,I5:I171)</f>
-        <v>25.3098499498091</v>
+        <v>23.2698499498091</v>
       </c>
       <c r="J172" s="12" t="n">
         <f aca="false">SUBTOTAL(9,J5:J171)</f>
@@ -13486,11 +13486,11 @@
       </c>
       <c r="K172" s="12" t="n">
         <f aca="false">SUBTOTAL(9,K5:K171)</f>
-        <v>1997.16039909105</v>
+        <v>1998.76556397618</v>
       </c>
       <c r="L172" s="12" t="n">
         <f aca="false">SUBTOTAL(9,L5:L171)</f>
-        <v>315.051592890545</v>
+        <v>313.446428005422</v>
       </c>
       <c r="M172" s="12" t="n">
         <f aca="false">SUBTOTAL(9,M5:M171)</f>
@@ -13615,7 +13615,7 @@
       </c>
       <c r="B4" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A4,'Plant x size'!$C$5:$C$171)</f>
-        <v>12.3127576</v>
+        <v>8.21275760000001</v>
       </c>
       <c r="C4" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A4,'Plant x size'!$D$5:$D$171)</f>
@@ -14755,7 +14755,7 @@
       </c>
       <c r="B24" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A24,'Plant x size'!$C$5:$C$171)</f>
-        <v>33.9614816</v>
+        <v>27.9214816</v>
       </c>
       <c r="C24" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A24,'Plant x size'!$D$5:$D$171)</f>
@@ -14812,7 +14812,7 @@
       </c>
       <c r="B25" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A25,'Plant x size'!$C$5:$C$171)</f>
-        <v>23.10726</v>
+        <v>18.13226</v>
       </c>
       <c r="C25" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A25,'Plant x size'!$D$5:$D$171)</f>
@@ -15496,7 +15496,7 @@
       </c>
       <c r="B37" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A37,'Plant x size'!$C$5:$C$171)</f>
-        <v>30.9021872</v>
+        <v>27.7821872</v>
       </c>
       <c r="C37" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A37,'Plant x size'!$D$5:$D$171)</f>
@@ -15553,7 +15553,7 @@
       </c>
       <c r="B38" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A38,'Plant x size'!$C$5:$C$171)</f>
-        <v>6.94151360000002</v>
+        <v>4.94651360000001</v>
       </c>
       <c r="C38" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A38,'Plant x size'!$D$5:$D$171)</f>
@@ -15610,7 +15610,7 @@
       </c>
       <c r="B39" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A39,'Plant x size'!$C$5:$C$171)</f>
-        <v>22.16657</v>
+        <v>16.99157</v>
       </c>
       <c r="C39" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A39,'Plant x size'!$D$5:$D$171)</f>
@@ -15618,11 +15618,11 @@
       </c>
       <c r="D39" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A39,'Plant x size'!$K$5:$K$171)</f>
-        <v>19.9741088766377</v>
+        <v>20</v>
       </c>
       <c r="E39" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A39,'Plant x size'!$L$5:$L$171)</f>
-        <v>8.32589112336227</v>
+        <v>8.3</v>
       </c>
       <c r="F39" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A39,'Plant x size'!$M$5:$M$171)</f>
@@ -16294,7 +16294,7 @@
       </c>
       <c r="B51" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A51,'Plant x size'!$C$5:$C$171)</f>
-        <v>11.3509284</v>
+        <v>7.2709284</v>
       </c>
       <c r="C51" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A51,'Plant x size'!$D$5:$D$171)</f>
@@ -16522,7 +16522,7 @@
       </c>
       <c r="B55" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A55,'Plant x size'!$C$5:$C$171)</f>
-        <v>63.6501984</v>
+        <v>59.6501984</v>
       </c>
       <c r="C55" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A55,'Plant x size'!$D$5:$D$171)</f>
@@ -16978,7 +16978,7 @@
       </c>
       <c r="B63" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A63,'Plant x size'!$C$5:$C$171)</f>
-        <v>152.523296</v>
+        <v>146.523296</v>
       </c>
       <c r="C63" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A63,'Plant x size'!$D$5:$D$171)</f>
@@ -17035,7 +17035,7 @@
       </c>
       <c r="B64" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A64,'Plant x size'!$C$5:$C$171)</f>
-        <v>102.231245</v>
+        <v>100.331245</v>
       </c>
       <c r="C64" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A64,'Plant x size'!$D$5:$D$171)</f>
@@ -17043,11 +17043,11 @@
       </c>
       <c r="D64" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A64,'Plant x size'!$K$5:$K$171)</f>
-        <v>95.6622067871455</v>
+        <v>97.2414805489063</v>
       </c>
       <c r="E64" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A64,'Plant x size'!$L$5:$L$171)</f>
-        <v>2.22179321285452</v>
+        <v>0.642519451093735</v>
       </c>
       <c r="F64" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A64,'Plant x size'!$M$5:$M$171)</f>
@@ -17662,7 +17662,7 @@
       </c>
       <c r="B75" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A75,'Plant x size'!$C$5:$C$171)</f>
-        <v>12.3371932480001</v>
+        <v>6.18719324800005</v>
       </c>
       <c r="C75" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A75,'Plant x size'!$D$5:$D$171)</f>
@@ -17890,7 +17890,7 @@
       </c>
       <c r="B79" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A79,'Plant x size'!$C$5:$C$171)</f>
-        <v>58.8083268</v>
+        <v>54.9333268</v>
       </c>
       <c r="C79" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A79,'Plant x size'!$D$5:$D$171)</f>
@@ -18745,7 +18745,7 @@
       </c>
       <c r="B94" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A94,'Plant x size'!$C$5:$C$171)</f>
-        <v>9.04905037447167</v>
+        <v>7.00905037447168</v>
       </c>
       <c r="C94" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A94,'Plant x size'!$D$5:$D$171)</f>
@@ -20170,7 +20170,7 @@
       </c>
       <c r="B119" s="12" t="n">
         <f aca="false">SUBTOTAL(9,B4:B118)</f>
-        <v>2573.49662731872</v>
+        <v>2520.04662731872</v>
       </c>
       <c r="C119" s="12" t="n">
         <f aca="false">SUBTOTAL(9,C4:C118)</f>
@@ -20178,11 +20178,11 @@
       </c>
       <c r="D119" s="12" t="n">
         <f aca="false">SUBTOTAL(9,D4:D118)</f>
-        <v>1997.16039909105</v>
+        <v>1998.76556397618</v>
       </c>
       <c r="E119" s="12" t="n">
         <f aca="false">SUBTOTAL(9,E4:E118)</f>
-        <v>315.051592890545</v>
+        <v>313.446428005422</v>
       </c>
       <c r="F119" s="12" t="n">
         <f aca="false">SUBTOTAL(9,F4:F118)</f>

</xml_diff>

<commit_message>
Calibrated FG ageing: exclude invoices dated 29-Oct (user decision)
The plants' 29-Oct FG sheets were counted before those invoices (Hyderabad
28.27 MT, Tapi 25.18 MT). Figures equal the build verified on pre-12:36 data.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SVVKmwQKKV189dev92iFna
</commit_message>
<xml_diff>
--- a/reports/FG-Ageing-Calibrated-2026-10-29.xlsx
+++ b/reports/FG-Ageing-Calibrated-2026-10-29.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="159">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="518" uniqueCount="160">
   <si>
     <t xml:space="preserve">FG ageing calibrated to plant FG sheets - by plant (29-Oct-2026)</t>
   </si>
@@ -101,6 +101,9 @@
     <t xml:space="preserve">Tapi: the sheet shows whole tonnes; its rows add to 827 against a printed 826 (rounding). Lepakshi's sheet is not titled; it is identified as Lepakshi from its sizes.</t>
   </si>
   <si>
+    <t xml:space="preserve">Invoices dated 29-Oct (Hyderabad 28.27 MT, Tapi 25.18 MT) are left out, as decided on 29-Oct: the plant sheets of 29-Oct are counted before them.</t>
+  </si>
+  <si>
     <t xml:space="preserve">NPMD: HR and CRFH lines of the same size are added together (the system does not split them). Hyderabad's "25.4OD" rows are matched to CHS 20 NB.</t>
   </si>
   <si>
@@ -119,7 +122,7 @@
     <t xml:space="preserve">FG ageing calibrated to plant FG sheets - by plant and size (29-Oct-2026)</t>
   </si>
   <si>
-    <t xml:space="preserve">System FG and FIFO ageing from the database (production to 26-28 Oct and invoices to 24-29 Oct, by plant). Thickness clubbed to 1.6 / 2 / 2.5 / 3 / 4 / 5 / 6. Each size is calibrated to the plant sheet: ratio = plant FG / system FG, and every age bucket is multiplied by it. Plant stock the system shows as nil is "Age unknown".</t>
+    <t xml:space="preserve">System FG and FIFO ageing from the database (production to 26-28 Oct and invoices to 24-28 Oct, by plant; invoices dated 29-Oct excluded). Thickness clubbed to 1.6 / 2 / 2.5 / 3 / 4 / 5 / 6. Each size is calibrated to the plant sheet: ratio = plant FG / system FG, and every age bucket is multiplied by it. Plant stock the system shows as nil is "Age unknown".</t>
   </si>
   <si>
     <t xml:space="preserve">Size</t>
@@ -1178,7 +1181,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:N18"/>
+  <dimension ref="A1:N19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
@@ -1248,7 +1251,7 @@
       </c>
       <c r="B4" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$A$5:$A$171,A4,'Plant x size'!$C$5:$C$171)</f>
-        <v>655.15496592272</v>
+        <v>683.42496592272</v>
       </c>
       <c r="C4" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$A$5:$A$171,A4,'Plant x size'!$D$5:$D$171)</f>
@@ -1256,15 +1259,15 @@
       </c>
       <c r="D4" s="9" t="n">
         <f aca="false">IF(B4&gt;0,C4/B4,0)</f>
-        <v>0.982106575493618</v>
+        <v>0.941481555522744</v>
       </c>
       <c r="E4" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$A$5:$A$171,A4,'Plant x size'!$K$5:$K$171)</f>
-        <v>326.85578916002</v>
+        <v>325.276515398259</v>
       </c>
       <c r="F4" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$A$5:$A$171,A4,'Plant x size'!$L$5:$L$171)</f>
-        <v>87.6562028215772</v>
+        <v>89.235476583338</v>
       </c>
       <c r="G4" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$A$5:$A$171,A4,'Plant x size'!$M$5:$M$171)</f>
@@ -1292,7 +1295,7 @@
       </c>
       <c r="M4" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$A$5:$A$171,A4,'Plant x size'!$I$5:$I$171)+SUMIF('Plant x size'!$A$5:$A$171,A4,'Plant x size'!$J$5:$J$171)</f>
-        <v>239.037166636955</v>
+        <v>241.077166636955</v>
       </c>
       <c r="N4" s="8" t="n">
         <v>649.586</v>
@@ -1416,7 +1419,7 @@
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$A$5:$A$171,A7,'Plant x size'!$C$5:$C$171)</f>
-        <v>759.5845037</v>
+        <v>784.7645037</v>
       </c>
       <c r="C7" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$A$5:$A$171,A7,'Plant x size'!$D$5:$D$171)</f>
@@ -1424,15 +1427,15 @@
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">IF(B7&gt;0,C7/B7,0)</f>
-        <v>1.08875312222882</v>
+        <v>1.05381932554399</v>
       </c>
       <c r="E7" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$A$5:$A$171,A7,'Plant x size'!$K$5:$K$171)</f>
-        <v>731.365841853333</v>
+        <v>731.339950729971</v>
       </c>
       <c r="F7" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$A$5:$A$171,A7,'Plant x size'!$L$5:$L$171)</f>
-        <v>24.6341581466672</v>
+        <v>24.6600492700294</v>
       </c>
       <c r="G7" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$A$5:$A$171,A7,'Plant x size'!$M$5:$M$171)</f>
@@ -1472,7 +1475,7 @@
       </c>
       <c r="B8" s="12" t="n">
         <f aca="false">SUM(B4:B7)</f>
-        <v>2520.04662731872</v>
+        <v>2573.49662731872</v>
       </c>
       <c r="C8" s="12" t="n">
         <f aca="false">SUM(C4:C7)</f>
@@ -1480,15 +1483,15 @@
       </c>
       <c r="D8" s="13" t="n">
         <f aca="false">IF(B8&gt;0,C8/B8,0)</f>
-        <v>1.0439219542533</v>
+        <v>1.02224031384914</v>
       </c>
       <c r="E8" s="12" t="n">
         <f aca="false">SUM(E4:E7)</f>
-        <v>1998.76556397618</v>
+        <v>1997.16039909105</v>
       </c>
       <c r="F8" s="12" t="n">
         <f aca="false">SUM(F4:F7)</f>
-        <v>313.446428005422</v>
+        <v>315.051592890545</v>
       </c>
       <c r="G8" s="12" t="n">
         <f aca="false">SUM(G4:G7)</f>
@@ -1516,7 +1519,7 @@
       </c>
       <c r="M8" s="12" t="n">
         <f aca="false">SUM(M4:M7)</f>
-        <v>243.531414636955</v>
+        <v>245.571414636955</v>
       </c>
       <c r="N8" s="12" t="n">
         <f aca="false">SUM(N4:N7)</f>
@@ -1566,6 +1569,11 @@
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="16" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -1602,12 +1610,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1615,31 +1623,31 @@
         <v>1</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>2</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="K4" s="3" t="s">
         <v>5</v>
@@ -1663,13 +1671,13 @@
         <v>11</v>
       </c>
       <c r="R4" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="S4" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="T4" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1677,24 +1685,24 @@
         <v>15</v>
       </c>
       <c r="B5" s="19" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C5" s="8" t="n">
-        <v>8.21275760000001</v>
+        <v>12.3127576</v>
       </c>
       <c r="D5" s="8" t="n">
         <v>11.749</v>
       </c>
       <c r="E5" s="20" t="n">
         <f aca="false">IF(C5&gt;0,D5/C5,"")</f>
-        <v>1.43057917598834</v>
+        <v>0.954213538647101</v>
       </c>
       <c r="F5" s="18" t="str">
         <f aca="false">IF(AND(C5=0,D5&gt;0),"Plant only",IF(AND(D5=0,C5&gt;0),"System only",IF(ABS(D5-C5)&lt;=0.5,"Match",IF(D5&gt;C5,"Plant more","Plant less"))))</f>
-        <v>Plant more</v>
+        <v>Plant less</v>
       </c>
       <c r="G5" s="8" t="n">
-        <v>8.21275760000001</v>
+        <v>12.3127576</v>
       </c>
       <c r="H5" s="8" t="n">
         <v>0</v>
@@ -1734,10 +1742,10 @@
         <v>0</v>
       </c>
       <c r="R5" s="21" t="n">
-        <v>9</v>
+        <v>11.4840348030566</v>
       </c>
       <c r="S5" s="22" t="n">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="T5" s="23" t="n">
         <v>46315</v>
@@ -1748,7 +1756,7 @@
         <v>15</v>
       </c>
       <c r="B6" s="19" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C6" s="8" t="n">
         <v>0</v>
@@ -1815,7 +1823,7 @@
         <v>15</v>
       </c>
       <c r="B7" s="19" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C7" s="8" t="n">
         <v>0.398907968</v>
@@ -1886,7 +1894,7 @@
         <v>15</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C8" s="8" t="n">
         <v>3.4545625</v>
@@ -1957,7 +1965,7 @@
         <v>15</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C9" s="8" t="n">
         <v>1.1760019200002</v>
@@ -2028,7 +2036,7 @@
         <v>15</v>
       </c>
       <c r="B10" s="19" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C10" s="8" t="n">
         <v>31.996960096</v>
@@ -2099,7 +2107,7 @@
         <v>15</v>
       </c>
       <c r="B11" s="19" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C11" s="8" t="n">
         <v>23.161798</v>
@@ -2170,7 +2178,7 @@
         <v>15</v>
       </c>
       <c r="B12" s="19" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C12" s="8" t="n">
         <v>8.127012416</v>
@@ -2241,7 +2249,7 @@
         <v>15</v>
       </c>
       <c r="B13" s="19" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C13" s="8" t="n">
         <v>0.0619999999999976</v>
@@ -2312,7 +2320,7 @@
         <v>15</v>
       </c>
       <c r="B14" s="19" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C14" s="8" t="n">
         <v>7.27215641600006</v>
@@ -2383,7 +2391,7 @@
         <v>15</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C15" s="8" t="n">
         <v>6.120127152</v>
@@ -2454,7 +2462,7 @@
         <v>15</v>
       </c>
       <c r="B16" s="19" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C16" s="8" t="n">
         <v>0.919102499999987</v>
@@ -2525,7 +2533,7 @@
         <v>15</v>
       </c>
       <c r="B17" s="19" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C17" s="8" t="n">
         <v>0.729902816000028</v>
@@ -2596,7 +2604,7 @@
         <v>15</v>
       </c>
       <c r="B18" s="19" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C18" s="8" t="n">
         <v>0.992313599999996</v>
@@ -2667,7 +2675,7 @@
         <v>15</v>
       </c>
       <c r="B19" s="19" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C19" s="8" t="n">
         <v>2.4611925</v>
@@ -2738,7 +2746,7 @@
         <v>15</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C20" s="8" t="n">
         <v>2.7322976</v>
@@ -2809,7 +2817,7 @@
         <v>15</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C21" s="8" t="n">
         <v>0.810000000000002</v>
@@ -2880,7 +2888,7 @@
         <v>15</v>
       </c>
       <c r="B22" s="19" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C22" s="8" t="n">
         <v>0.365000000000002</v>
@@ -2951,7 +2959,7 @@
         <v>15</v>
       </c>
       <c r="B23" s="19" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C23" s="8" t="n">
         <v>1.83006536000001</v>
@@ -3022,7 +3030,7 @@
         <v>15</v>
       </c>
       <c r="B24" s="19" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C24" s="8" t="n">
         <v>0</v>
@@ -3089,7 +3097,7 @@
         <v>15</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C25" s="8" t="n">
         <v>10.190473856</v>
@@ -3160,24 +3168,24 @@
         <v>15</v>
       </c>
       <c r="B26" s="19" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C26" s="8" t="n">
-        <v>7.2709284</v>
+        <v>11.3509284</v>
       </c>
       <c r="D26" s="8" t="n">
         <v>16.866</v>
       </c>
       <c r="E26" s="20" t="n">
         <f aca="false">IF(C26&gt;0,D26/C26,"")</f>
-        <v>2.31964875352094</v>
+        <v>1.48586964921742</v>
       </c>
       <c r="F26" s="18" t="str">
         <f aca="false">IF(AND(C26=0,D26&gt;0),"Plant only",IF(AND(D26=0,C26&gt;0),"System only",IF(ABS(D26-C26)&lt;=0.5,"Match",IF(D26&gt;C26,"Plant more","Plant less"))))</f>
         <v>Plant more</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>7.2709284</v>
+        <v>11.3509284</v>
       </c>
       <c r="H26" s="8" t="n">
         <v>0</v>
@@ -3231,7 +3239,7 @@
         <v>15</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C27" s="8" t="n">
         <v>1.93852</v>
@@ -3302,7 +3310,7 @@
         <v>15</v>
       </c>
       <c r="B28" s="19" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C28" s="8" t="n">
         <v>1.49284396800001</v>
@@ -3373,7 +3381,7 @@
         <v>15</v>
       </c>
       <c r="B29" s="19" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C29" s="8" t="n">
         <v>0.480092352000177</v>
@@ -3444,24 +3452,24 @@
         <v>15</v>
       </c>
       <c r="B30" s="19" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C30" s="8" t="n">
-        <v>16.6869648</v>
+        <v>20.6869648</v>
       </c>
       <c r="D30" s="8" t="n">
         <v>22.891</v>
       </c>
       <c r="E30" s="20" t="n">
         <f aca="false">IF(C30&gt;0,D30/C30,"")</f>
-        <v>1.37178931425564</v>
+        <v>1.10654222218235</v>
       </c>
       <c r="F30" s="18" t="str">
         <f aca="false">IF(AND(C30=0,D30&gt;0),"Plant only",IF(AND(D30=0,C30&gt;0),"System only",IF(ABS(D30-C30)&lt;=0.5,"Match",IF(D30&gt;C30,"Plant more","Plant less"))))</f>
         <v>Plant more</v>
       </c>
       <c r="G30" s="8" t="n">
-        <v>16.6869648</v>
+        <v>20.6869648</v>
       </c>
       <c r="H30" s="8" t="n">
         <v>0</v>
@@ -3515,7 +3523,7 @@
         <v>15</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C31" s="8" t="n">
         <v>13.0084675</v>
@@ -3586,7 +3594,7 @@
         <v>15</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C32" s="8" t="n">
         <v>22.624130496</v>
@@ -3657,7 +3665,7 @@
         <v>15</v>
       </c>
       <c r="B33" s="19" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C33" s="8" t="n">
         <v>9.59333920000001</v>
@@ -3728,7 +3736,7 @@
         <v>15</v>
       </c>
       <c r="B34" s="19" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C34" s="8" t="n">
         <v>1.095805</v>
@@ -3799,7 +3807,7 @@
         <v>15</v>
       </c>
       <c r="B35" s="19" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C35" s="8" t="n">
         <v>20.02434368</v>
@@ -3870,24 +3878,24 @@
         <v>15</v>
       </c>
       <c r="B36" s="19" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C36" s="8" t="n">
-        <v>29.7587936</v>
+        <v>35.7587936</v>
       </c>
       <c r="D36" s="8" t="n">
         <v>28.752</v>
       </c>
       <c r="E36" s="20" t="n">
         <f aca="false">IF(C36&gt;0,D36/C36,"")</f>
-        <v>0.966168198431271</v>
+        <v>0.804053971216748</v>
       </c>
       <c r="F36" s="18" t="str">
         <f aca="false">IF(AND(C36=0,D36&gt;0),"Plant only",IF(AND(D36=0,C36&gt;0),"System only",IF(ABS(D36-C36)&lt;=0.5,"Match",IF(D36&gt;C36,"Plant more","Plant less"))))</f>
         <v>Plant less</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>29.7587936</v>
+        <v>35.7587936</v>
       </c>
       <c r="H36" s="8" t="n">
         <v>0</v>
@@ -3941,17 +3949,17 @@
         <v>15</v>
       </c>
       <c r="B37" s="19" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C37" s="8" t="n">
-        <v>20.046045</v>
+        <v>21.946045</v>
       </c>
       <c r="D37" s="8" t="n">
         <v>18.884</v>
       </c>
       <c r="E37" s="20" t="n">
         <f aca="false">IF(C37&gt;0,D37/C37,"")</f>
-        <v>0.942031208649885</v>
+        <v>0.86047394872288</v>
       </c>
       <c r="F37" s="18" t="str">
         <f aca="false">IF(AND(C37=0,D37&gt;0),"Plant only",IF(AND(D37=0,C37&gt;0),"System only",IF(ABS(D37-C37)&lt;=0.5,"Match",IF(D37&gt;C37,"Plant more","Plant less"))))</f>
@@ -3961,7 +3969,7 @@
         <v>19.3639875</v>
       </c>
       <c r="H37" s="8" t="n">
-        <v>0.682057500000017</v>
+        <v>2.58205749999999</v>
       </c>
       <c r="I37" s="8" t="n">
         <v>0</v>
@@ -3971,11 +3979,11 @@
       </c>
       <c r="K37" s="8" t="n">
         <f aca="false">IF(C37&gt;0,G37*E37,0)</f>
-        <v>18.2414805489063</v>
+        <v>16.6622067871455</v>
       </c>
       <c r="L37" s="8" t="n">
         <f aca="false">IF(C37&gt;0,H37*E37,0)</f>
-        <v>0.642519451093735</v>
+        <v>2.22179321285452</v>
       </c>
       <c r="M37" s="8" t="n">
         <f aca="false">IF(C37&gt;0,I37*E37,0)</f>
@@ -3998,7 +4006,7 @@
         <v>0</v>
       </c>
       <c r="R37" s="21" t="n">
-        <v>5.15232194180951</v>
+        <v>8.77532500730769</v>
       </c>
       <c r="S37" s="22" t="n">
         <v>47</v>
@@ -4012,7 +4020,7 @@
         <v>15</v>
       </c>
       <c r="B38" s="19" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C38" s="8" t="n">
         <v>24.529190656</v>
@@ -4083,7 +4091,7 @@
         <v>15</v>
       </c>
       <c r="B39" s="19" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C39" s="8" t="n">
         <v>22.1014464</v>
@@ -4154,7 +4162,7 @@
         <v>15</v>
       </c>
       <c r="B40" s="19" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C40" s="8" t="n">
         <v>3.09150749999996</v>
@@ -4225,24 +4233,24 @@
         <v>15</v>
       </c>
       <c r="B41" s="19" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C41" s="8" t="n">
-        <v>6.18719324800005</v>
+        <v>12.3371932480001</v>
       </c>
       <c r="D41" s="8" t="n">
         <v>8.726</v>
       </c>
       <c r="E41" s="20" t="n">
         <f aca="false">IF(C41&gt;0,D41/C41,"")</f>
-        <v>1.41033254502283</v>
+        <v>0.707292155078672</v>
       </c>
       <c r="F41" s="18" t="str">
         <f aca="false">IF(AND(C41=0,D41&gt;0),"Plant only",IF(AND(D41=0,C41&gt;0),"System only",IF(ABS(D41-C41)&lt;=0.5,"Match",IF(D41&gt;C41,"Plant more","Plant less"))))</f>
-        <v>Plant more</v>
+        <v>Plant less</v>
       </c>
       <c r="G41" s="8" t="n">
-        <v>6.18719324800005</v>
+        <v>12.3371932480001</v>
       </c>
       <c r="H41" s="8" t="n">
         <v>0</v>
@@ -4296,7 +4304,7 @@
         <v>15</v>
       </c>
       <c r="B42" s="19" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C42" s="8" t="n">
         <v>14.6710672</v>
@@ -4367,7 +4375,7 @@
         <v>15</v>
       </c>
       <c r="B43" s="19" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C43" s="8" t="n">
         <v>3.38020000000001</v>
@@ -4438,7 +4446,7 @@
         <v>15</v>
       </c>
       <c r="B44" s="19" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C44" s="8" t="n">
         <v>5.2602</v>
@@ -4509,7 +4517,7 @@
         <v>15</v>
       </c>
       <c r="B45" s="19" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C45" s="8" t="n">
         <v>20.3448108030086</v>
@@ -4580,7 +4588,7 @@
         <v>15</v>
       </c>
       <c r="B46" s="19" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C46" s="8" t="n">
         <v>14.6224114638618</v>
@@ -4651,7 +4659,7 @@
         <v>15</v>
       </c>
       <c r="B47" s="19" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C47" s="8" t="n">
         <v>10.6181676337717</v>
@@ -4722,7 +4730,7 @@
         <v>15</v>
       </c>
       <c r="B48" s="19" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C48" s="8" t="n">
         <v>9.69094282016051</v>
@@ -4793,21 +4801,21 @@
         <v>15</v>
       </c>
       <c r="B49" s="19" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C49" s="8" t="n">
-        <v>7.00905037447168</v>
+        <v>9.04905037447167</v>
       </c>
       <c r="D49" s="8" t="n">
         <v>6.762</v>
       </c>
       <c r="E49" s="20" t="n">
         <f aca="false">IF(C49&gt;0,D49/C49,"")</f>
-        <v>0.964752661020745</v>
+        <v>0.747260731255991</v>
       </c>
       <c r="F49" s="18" t="str">
         <f aca="false">IF(AND(C49=0,D49&gt;0),"Plant only",IF(AND(D49=0,C49&gt;0),"System only",IF(ABS(D49-C49)&lt;=0.5,"Match",IF(D49&gt;C49,"Plant more","Plant less"))))</f>
-        <v>Match</v>
+        <v>Plant less</v>
       </c>
       <c r="G49" s="8" t="n">
         <v>0</v>
@@ -4816,7 +4824,7 @@
         <v>0</v>
       </c>
       <c r="I49" s="8" t="n">
-        <v>7.00905037447168</v>
+        <v>9.04905037447167</v>
       </c>
       <c r="J49" s="8" t="n">
         <v>0</v>
@@ -4864,7 +4872,7 @@
         <v>15</v>
       </c>
       <c r="B50" s="19" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C50" s="8" t="n">
         <v>0.884169445298547</v>
@@ -4935,7 +4943,7 @@
         <v>15</v>
       </c>
       <c r="B51" s="19" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C51" s="8" t="n">
         <v>0.27654390180969</v>
@@ -5006,7 +5014,7 @@
         <v>15</v>
       </c>
       <c r="B52" s="19" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C52" s="8" t="n">
         <v>0</v>
@@ -5073,7 +5081,7 @@
         <v>15</v>
       </c>
       <c r="B53" s="19" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C53" s="8" t="n">
         <v>1.35044088702466</v>
@@ -5144,7 +5152,7 @@
         <v>15</v>
       </c>
       <c r="B54" s="19" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C54" s="8" t="n">
         <v>7.39196666203889</v>
@@ -5215,7 +5223,7 @@
         <v>15</v>
       </c>
       <c r="B55" s="19" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C55" s="8" t="n">
         <v>25.7355663919971</v>
@@ -5286,7 +5294,7 @@
         <v>15</v>
       </c>
       <c r="B56" s="19" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C56" s="8" t="n">
         <v>2.36277335267008</v>
@@ -5357,7 +5365,7 @@
         <v>15</v>
       </c>
       <c r="B57" s="19" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C57" s="8" t="n">
         <v>24.6311525361491</v>
@@ -5428,7 +5436,7 @@
         <v>15</v>
       </c>
       <c r="B58" s="19" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C58" s="8" t="n">
         <v>1.10166481737043</v>
@@ -5499,7 +5507,7 @@
         <v>15</v>
       </c>
       <c r="B59" s="19" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C59" s="8" t="n">
         <v>0.243142977051814</v>
@@ -5570,7 +5578,7 @@
         <v>15</v>
       </c>
       <c r="B60" s="19" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C60" s="8" t="n">
         <v>6.987</v>
@@ -5641,7 +5649,7 @@
         <v>15</v>
       </c>
       <c r="B61" s="19" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C61" s="8" t="n">
         <v>1.6796943760219</v>
@@ -5712,7 +5720,7 @@
         <v>15</v>
       </c>
       <c r="B62" s="19" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C62" s="8" t="n">
         <v>32.8148270267837</v>
@@ -5783,7 +5791,7 @@
         <v>15</v>
       </c>
       <c r="B63" s="19" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C63" s="8" t="n">
         <v>14.0415575471577</v>
@@ -5854,7 +5862,7 @@
         <v>15</v>
       </c>
       <c r="B64" s="19" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C64" s="8" t="n">
         <v>18.6965553667495</v>
@@ -5925,7 +5933,7 @@
         <v>15</v>
       </c>
       <c r="B65" s="19" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C65" s="8" t="n">
         <v>10.1022607216639</v>
@@ -5996,7 +6004,7 @@
         <v>15</v>
       </c>
       <c r="B66" s="19" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C66" s="8" t="n">
         <v>5.43362912409522</v>
@@ -6067,7 +6075,7 @@
         <v>15</v>
       </c>
       <c r="B67" s="19" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C67" s="8" t="n">
         <v>5.38384355438487</v>
@@ -6138,7 +6146,7 @@
         <v>15</v>
       </c>
       <c r="B68" s="19" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C68" s="8" t="n">
         <v>0.0172000000000008</v>
@@ -6209,7 +6217,7 @@
         <v>15</v>
       </c>
       <c r="B69" s="19" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C69" s="8" t="n">
         <v>15.21</v>
@@ -6280,7 +6288,7 @@
         <v>15</v>
       </c>
       <c r="B70" s="19" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="C70" s="8" t="n">
         <v>16.9689453224326</v>
@@ -6351,7 +6359,7 @@
         <v>15</v>
       </c>
       <c r="B71" s="19" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C71" s="8" t="n">
         <v>34.3465701717689</v>
@@ -6422,7 +6430,7 @@
         <v>15</v>
       </c>
       <c r="B72" s="19" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C72" s="8" t="n">
         <v>13.3602673449761</v>
@@ -6493,7 +6501,7 @@
         <v>15</v>
       </c>
       <c r="B73" s="19" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C73" s="8" t="n">
         <v>19.5961</v>
@@ -6564,7 +6572,7 @@
         <v>16</v>
       </c>
       <c r="B74" s="19" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C74" s="8" t="n">
         <v>0</v>
@@ -6629,7 +6637,7 @@
         <v>16</v>
       </c>
       <c r="B75" s="19" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C75" s="8" t="n">
         <v>0</v>
@@ -6694,7 +6702,7 @@
         <v>16</v>
       </c>
       <c r="B76" s="19" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C76" s="8" t="n">
         <v>5.55292480000001</v>
@@ -6765,7 +6773,7 @@
         <v>16</v>
       </c>
       <c r="B77" s="19" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C77" s="8" t="n">
         <v>6.5123125</v>
@@ -6836,7 +6844,7 @@
         <v>16</v>
       </c>
       <c r="B78" s="19" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C78" s="8" t="n">
         <v>4.667348</v>
@@ -6907,7 +6915,7 @@
         <v>16</v>
       </c>
       <c r="B79" s="19" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C79" s="8" t="n">
         <v>1.86896</v>
@@ -6978,7 +6986,7 @@
         <v>16</v>
       </c>
       <c r="B80" s="19" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C80" s="8" t="n">
         <v>5.3884585</v>
@@ -7049,7 +7057,7 @@
         <v>16</v>
       </c>
       <c r="B81" s="19" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C81" s="8" t="n">
         <v>0</v>
@@ -7116,7 +7124,7 @@
         <v>16</v>
       </c>
       <c r="B82" s="19" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C82" s="8" t="n">
         <v>51.75348</v>
@@ -7187,7 +7195,7 @@
         <v>16</v>
       </c>
       <c r="B83" s="19" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C83" s="8" t="n">
         <v>0.333020799999996</v>
@@ -7258,7 +7266,7 @@
         <v>16</v>
       </c>
       <c r="B84" s="19" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C84" s="8" t="n">
         <v>0.267739999999995</v>
@@ -7329,7 +7337,7 @@
         <v>16</v>
       </c>
       <c r="B85" s="19" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C85" s="8" t="n">
         <v>0.535804799999998</v>
@@ -7400,7 +7408,7 @@
         <v>16</v>
       </c>
       <c r="B86" s="19" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C86" s="8" t="n">
         <v>0</v>
@@ -7467,7 +7475,7 @@
         <v>16</v>
       </c>
       <c r="B87" s="19" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C87" s="8" t="n">
         <v>2.00522</v>
@@ -7538,7 +7546,7 @@
         <v>16</v>
       </c>
       <c r="B88" s="19" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C88" s="8" t="n">
         <v>37.7925888</v>
@@ -7609,7 +7617,7 @@
         <v>16</v>
       </c>
       <c r="B89" s="19" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C89" s="8" t="n">
         <v>35.024976</v>
@@ -7680,7 +7688,7 @@
         <v>16</v>
       </c>
       <c r="B90" s="19" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C90" s="8" t="n">
         <v>41.17071</v>
@@ -7751,7 +7759,7 @@
         <v>16</v>
       </c>
       <c r="B91" s="19" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C91" s="8" t="n">
         <v>0</v>
@@ -7816,7 +7824,7 @@
         <v>16</v>
       </c>
       <c r="B92" s="19" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C92" s="8" t="n">
         <v>6.1211178</v>
@@ -7887,7 +7895,7 @@
         <v>16</v>
       </c>
       <c r="B93" s="19" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C93" s="8" t="n">
         <v>3.771654</v>
@@ -7958,7 +7966,7 @@
         <v>16</v>
       </c>
       <c r="B94" s="19" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C94" s="8" t="n">
         <v>8.3800532</v>
@@ -8029,7 +8037,7 @@
         <v>16</v>
       </c>
       <c r="B95" s="19" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C95" s="8" t="n">
         <v>4.2607808</v>
@@ -8100,7 +8108,7 @@
         <v>16</v>
       </c>
       <c r="B96" s="19" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C96" s="8" t="n">
         <v>22.771162</v>
@@ -8171,7 +8179,7 @@
         <v>16</v>
       </c>
       <c r="B97" s="19" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C97" s="8" t="n">
         <v>2.392126</v>
@@ -8242,7 +8250,7 @@
         <v>16</v>
       </c>
       <c r="B98" s="19" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C98" s="8" t="n">
         <v>23.493792</v>
@@ -8313,7 +8321,7 @@
         <v>16</v>
       </c>
       <c r="B99" s="19" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C99" s="8" t="n">
         <v>9.700807</v>
@@ -8384,7 +8392,7 @@
         <v>16</v>
       </c>
       <c r="B100" s="19" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C100" s="8" t="n">
         <v>30.45868</v>
@@ -8455,7 +8463,7 @@
         <v>16</v>
       </c>
       <c r="B101" s="19" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C101" s="8" t="n">
         <v>23.196887</v>
@@ -8526,7 +8534,7 @@
         <v>17</v>
       </c>
       <c r="B102" s="19" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C102" s="8" t="n">
         <v>54.7693178240002</v>
@@ -8597,7 +8605,7 @@
         <v>17</v>
       </c>
       <c r="B103" s="19" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C103" s="8" t="n">
         <v>67.0330016</v>
@@ -8668,7 +8676,7 @@
         <v>17</v>
       </c>
       <c r="B104" s="19" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C104" s="8" t="n">
         <v>71.0481625</v>
@@ -8739,7 +8747,7 @@
         <v>17</v>
       </c>
       <c r="B105" s="19" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C105" s="8" t="n">
         <v>23.950528</v>
@@ -8810,7 +8818,7 @@
         <v>17</v>
       </c>
       <c r="B106" s="19" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C106" s="8" t="n">
         <v>29.997252</v>
@@ -8881,7 +8889,7 @@
         <v>17</v>
       </c>
       <c r="B107" s="19" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C107" s="8" t="n">
         <v>2.153178688</v>
@@ -8952,7 +8960,7 @@
         <v>17</v>
       </c>
       <c r="B108" s="19" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C108" s="8" t="n">
         <v>0</v>
@@ -9019,7 +9027,7 @@
         <v>17</v>
       </c>
       <c r="B109" s="19" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C109" s="8" t="n">
         <v>0</v>
@@ -9086,7 +9094,7 @@
         <v>17</v>
       </c>
       <c r="B110" s="19" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C110" s="8" t="n">
         <v>102.528854464</v>
@@ -9157,7 +9165,7 @@
         <v>17</v>
       </c>
       <c r="B111" s="19" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C111" s="8" t="n">
         <v>40.8825136</v>
@@ -9228,7 +9236,7 @@
         <v>17</v>
       </c>
       <c r="B112" s="19" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C112" s="8" t="n">
         <v>41.7639025</v>
@@ -9299,7 +9307,7 @@
         <v>17</v>
       </c>
       <c r="B113" s="19" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C113" s="8" t="n">
         <v>17.3729504</v>
@@ -9370,7 +9378,7 @@
         <v>17</v>
       </c>
       <c r="B114" s="19" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C114" s="8" t="n">
         <v>56.1601697920001</v>
@@ -9441,7 +9449,7 @@
         <v>17</v>
       </c>
       <c r="B115" s="19" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C115" s="8" t="n">
         <v>101.4804864</v>
@@ -9512,7 +9520,7 @@
         <v>17</v>
       </c>
       <c r="B116" s="19" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C116" s="8" t="n">
         <v>62.560575</v>
@@ -9583,7 +9591,7 @@
         <v>17</v>
       </c>
       <c r="B117" s="19" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C117" s="8" t="n">
         <v>28.7222888</v>
@@ -9654,7 +9662,7 @@
         <v>17</v>
       </c>
       <c r="B118" s="19" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C118" s="8" t="n">
         <v>19.777918528</v>
@@ -9725,7 +9733,7 @@
         <v>17</v>
       </c>
       <c r="B119" s="19" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C119" s="8" t="n">
         <v>40.21808</v>
@@ -9796,7 +9804,7 @@
         <v>17</v>
       </c>
       <c r="B120" s="19" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C120" s="8" t="n">
         <v>17.4673736</v>
@@ -9867,7 +9875,7 @@
         <v>18</v>
       </c>
       <c r="B121" s="19" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C121" s="8" t="n">
         <v>0.111864</v>
@@ -9938,7 +9946,7 @@
         <v>18</v>
       </c>
       <c r="B122" s="19" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C122" s="8" t="n">
         <v>0.0868599999999997</v>
@@ -10009,7 +10017,7 @@
         <v>18</v>
       </c>
       <c r="B123" s="19" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C123" s="8" t="n">
         <v>26.858584</v>
@@ -10080,7 +10088,7 @@
         <v>18</v>
       </c>
       <c r="B124" s="19" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C124" s="8" t="n">
         <v>7.1239375</v>
@@ -10151,7 +10159,7 @@
         <v>18</v>
       </c>
       <c r="B125" s="19" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C125" s="8" t="n">
         <v>4.432376</v>
@@ -10222,7 +10230,7 @@
         <v>18</v>
       </c>
       <c r="B126" s="19" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C126" s="8" t="n">
         <v>1.3121184</v>
@@ -10293,7 +10301,7 @@
         <v>18</v>
       </c>
       <c r="B127" s="19" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C127" s="8" t="n">
         <v>10.39302</v>
@@ -10364,24 +10372,24 @@
         <v>18</v>
       </c>
       <c r="B128" s="19" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C128" s="8" t="n">
-        <v>25.189184</v>
+        <v>31.229184</v>
       </c>
       <c r="D128" s="8" t="n">
         <v>33</v>
       </c>
       <c r="E128" s="20" t="n">
         <f aca="false">IF(C128&gt;0,D128/C128,"")</f>
-        <v>1.31008610679885</v>
+        <v>1.056703883137</v>
       </c>
       <c r="F128" s="18" t="str">
         <f aca="false">IF(AND(C128=0,D128&gt;0),"Plant only",IF(AND(D128=0,C128&gt;0),"System only",IF(ABS(D128-C128)&lt;=0.5,"Match",IF(D128&gt;C128,"Plant more","Plant less"))))</f>
         <v>Plant more</v>
       </c>
       <c r="G128" s="8" t="n">
-        <v>25.189184</v>
+        <v>31.229184</v>
       </c>
       <c r="H128" s="8" t="n">
         <v>0</v>
@@ -10435,24 +10443,24 @@
         <v>18</v>
       </c>
       <c r="B129" s="19" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C129" s="8" t="n">
-        <v>18.13226</v>
+        <v>23.10726</v>
       </c>
       <c r="D129" s="8" t="n">
         <v>23</v>
       </c>
       <c r="E129" s="20" t="n">
         <f aca="false">IF(C129&gt;0,D129/C129,"")</f>
-        <v>1.26845743442902</v>
+        <v>0.995358168817939</v>
       </c>
       <c r="F129" s="18" t="str">
         <f aca="false">IF(AND(C129=0,D129&gt;0),"Plant only",IF(AND(D129=0,C129&gt;0),"System only",IF(ABS(D129-C129)&lt;=0.5,"Match",IF(D129&gt;C129,"Plant more","Plant less"))))</f>
-        <v>Plant more</v>
+        <v>Match</v>
       </c>
       <c r="G129" s="8" t="n">
-        <v>18.13226</v>
+        <v>23.10726</v>
       </c>
       <c r="H129" s="8" t="n">
         <v>0</v>
@@ -10492,7 +10500,7 @@
         <v>0</v>
       </c>
       <c r="R129" s="21" t="n">
-        <v>1.21137464386679</v>
+        <v>1.38116591928251</v>
       </c>
       <c r="S129" s="22" t="n">
         <v>2</v>
@@ -10506,7 +10514,7 @@
         <v>18</v>
       </c>
       <c r="B130" s="19" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="C130" s="8" t="n">
         <v>0</v>
@@ -10573,7 +10581,7 @@
         <v>18</v>
       </c>
       <c r="B131" s="19" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C131" s="8" t="n">
         <v>31.238791</v>
@@ -10644,7 +10652,7 @@
         <v>18</v>
       </c>
       <c r="B132" s="19" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C132" s="8" t="n">
         <v>0</v>
@@ -10711,7 +10719,7 @@
         <v>18</v>
       </c>
       <c r="B133" s="19" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C133" s="8" t="n">
         <v>0</v>
@@ -10778,7 +10786,7 @@
         <v>18</v>
       </c>
       <c r="B134" s="19" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C134" s="8" t="n">
         <v>4.494248</v>
@@ -10849,7 +10857,7 @@
         <v>18</v>
       </c>
       <c r="B135" s="19" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C135" s="8" t="n">
         <v>0</v>
@@ -10916,7 +10924,7 @@
         <v>18</v>
       </c>
       <c r="B136" s="19" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C136" s="8" t="n">
         <v>5.0504</v>
@@ -10987,7 +10995,7 @@
         <v>18</v>
       </c>
       <c r="B137" s="19" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C137" s="8" t="n">
         <v>24.8301344</v>
@@ -11058,7 +11066,7 @@
         <v>18</v>
       </c>
       <c r="B138" s="19" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C138" s="8" t="n">
         <v>0.715932499999995</v>
@@ -11129,24 +11137,24 @@
         <v>18</v>
       </c>
       <c r="B139" s="19" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C139" s="8" t="n">
-        <v>27.2463824</v>
+        <v>30.3663824</v>
       </c>
       <c r="D139" s="8" t="n">
         <v>35</v>
       </c>
       <c r="E139" s="20" t="n">
         <f aca="false">IF(C139&gt;0,D139/C139,"")</f>
-        <v>1.28457420461074</v>
+        <v>1.15259037243765</v>
       </c>
       <c r="F139" s="18" t="str">
         <f aca="false">IF(AND(C139=0,D139&gt;0),"Plant only",IF(AND(D139=0,C139&gt;0),"System only",IF(ABS(D139-C139)&lt;=0.5,"Match",IF(D139&gt;C139,"Plant more","Plant less"))))</f>
         <v>Plant more</v>
       </c>
       <c r="G139" s="8" t="n">
-        <v>27.2463824</v>
+        <v>30.3663824</v>
       </c>
       <c r="H139" s="8" t="n">
         <v>0</v>
@@ -11186,7 +11194,7 @@
         <v>0</v>
       </c>
       <c r="R139" s="21" t="n">
-        <v>2.72202424935502</v>
+        <v>3.36705611663508</v>
       </c>
       <c r="S139" s="22" t="n">
         <v>9</v>
@@ -11200,24 +11208,24 @@
         <v>18</v>
       </c>
       <c r="B140" s="19" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C140" s="8" t="n">
-        <v>4.94651360000001</v>
+        <v>6.94151360000002</v>
       </c>
       <c r="D140" s="8" t="n">
         <v>12</v>
       </c>
       <c r="E140" s="20" t="n">
         <f aca="false">IF(C140&gt;0,D140/C140,"")</f>
-        <v>2.4259510779471</v>
+        <v>1.72872959580458</v>
       </c>
       <c r="F140" s="18" t="str">
         <f aca="false">IF(AND(C140=0,D140&gt;0),"Plant only",IF(AND(D140=0,C140&gt;0),"System only",IF(ABS(D140-C140)&lt;=0.5,"Match",IF(D140&gt;C140,"Plant more","Plant less"))))</f>
         <v>Plant more</v>
       </c>
       <c r="G140" s="8" t="n">
-        <v>4.94651360000001</v>
+        <v>6.94151360000002</v>
       </c>
       <c r="H140" s="8" t="n">
         <v>0</v>
@@ -11271,27 +11279,27 @@
         <v>18</v>
       </c>
       <c r="B141" s="19" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C141" s="8" t="n">
-        <v>14.98635</v>
+        <v>20.16135</v>
       </c>
       <c r="D141" s="8" t="n">
         <v>20</v>
       </c>
       <c r="E141" s="20" t="n">
         <f aca="false">IF(C141&gt;0,D141/C141,"")</f>
-        <v>1.33454777180568</v>
+        <v>0.991997063688692</v>
       </c>
       <c r="F141" s="18" t="str">
         <f aca="false">IF(AND(C141=0,D141&gt;0),"Plant only",IF(AND(D141=0,C141&gt;0),"System only",IF(ABS(D141-C141)&lt;=0.5,"Match",IF(D141&gt;C141,"Plant more","Plant less"))))</f>
-        <v>Plant more</v>
+        <v>Match</v>
       </c>
       <c r="G141" s="8" t="n">
-        <v>14.98635</v>
+        <v>20.13525</v>
       </c>
       <c r="H141" s="8" t="n">
-        <v>0</v>
+        <v>0.026099999999996</v>
       </c>
       <c r="I141" s="8" t="n">
         <v>0</v>
@@ -11301,11 +11309,11 @@
       </c>
       <c r="K141" s="8" t="n">
         <f aca="false">IF(C141&gt;0,G141*E141,0)</f>
-        <v>20</v>
+        <v>19.9741088766377</v>
       </c>
       <c r="L141" s="8" t="n">
         <f aca="false">IF(C141&gt;0,H141*E141,0)</f>
-        <v>0</v>
+        <v>0.0258911233622709</v>
       </c>
       <c r="M141" s="8" t="n">
         <f aca="false">IF(C141&gt;0,I141*E141,0)</f>
@@ -11328,10 +11336,10 @@
         <v>0</v>
       </c>
       <c r="R141" s="21" t="n">
-        <v>3</v>
+        <v>3.07378970158247</v>
       </c>
       <c r="S141" s="22" t="n">
-        <v>3</v>
+        <v>60</v>
       </c>
       <c r="T141" s="23" t="n">
         <v>46321</v>
@@ -11342,7 +11350,7 @@
         <v>18</v>
       </c>
       <c r="B142" s="19" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C142" s="8" t="n">
         <v>2.66855360000001</v>
@@ -11413,7 +11421,7 @@
         <v>18</v>
       </c>
       <c r="B143" s="19" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="C143" s="8" t="n">
         <v>0.762212000000002</v>
@@ -11484,7 +11492,7 @@
         <v>18</v>
       </c>
       <c r="B144" s="19" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C144" s="8" t="n">
         <v>0.0340639999999972</v>
@@ -11555,7 +11563,7 @@
         <v>18</v>
       </c>
       <c r="B145" s="19" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C145" s="8" t="n">
         <v>63.6940375</v>
@@ -11626,7 +11634,7 @@
         <v>18</v>
       </c>
       <c r="B146" s="19" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C146" s="8" t="n">
         <v>44.5940144</v>
@@ -11697,7 +11705,7 @@
         <v>18</v>
       </c>
       <c r="B147" s="19" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C147" s="8" t="n">
         <v>2.47299039999999</v>
@@ -11768,7 +11776,7 @@
         <v>18</v>
       </c>
       <c r="B148" s="19" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C148" s="8" t="n">
         <v>5.50399000000002</v>
@@ -11839,7 +11847,7 @@
         <v>18</v>
       </c>
       <c r="B149" s="19" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C149" s="8" t="n">
         <v>2.08072</v>
@@ -11910,7 +11918,7 @@
         <v>18</v>
       </c>
       <c r="B150" s="19" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C150" s="8" t="n">
         <v>0.152975000000001</v>
@@ -11981,7 +11989,7 @@
         <v>18</v>
       </c>
       <c r="B151" s="19" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C151" s="8" t="n">
         <v>3.8724</v>
@@ -12052,7 +12060,7 @@
         <v>18</v>
       </c>
       <c r="B152" s="19" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C152" s="8" t="n">
         <v>15.284016</v>
@@ -12123,7 +12131,7 @@
         <v>18</v>
       </c>
       <c r="B153" s="19" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C153" s="8" t="n">
         <v>17.724625</v>
@@ -12194,7 +12202,7 @@
         <v>18</v>
       </c>
       <c r="B154" s="19" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C154" s="8" t="n">
         <v>4.920268</v>
@@ -12265,7 +12273,7 @@
         <v>18</v>
       </c>
       <c r="B155" s="19" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C155" s="8" t="n">
         <v>42.2617312</v>
@@ -12336,7 +12344,7 @@
         <v>18</v>
       </c>
       <c r="B156" s="19" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C156" s="8" t="n">
         <v>52.94524</v>
@@ -12407,7 +12415,7 @@
         <v>18</v>
       </c>
       <c r="B157" s="19" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C157" s="8" t="n">
         <v>42.737136</v>
@@ -12478,7 +12486,7 @@
         <v>18</v>
       </c>
       <c r="B158" s="19" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C158" s="8" t="n">
         <v>40.37355</v>
@@ -12549,7 +12557,7 @@
         <v>18</v>
       </c>
       <c r="B159" s="19" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C159" s="8" t="n">
         <v>47.4872576</v>
@@ -12620,7 +12628,7 @@
         <v>18</v>
       </c>
       <c r="B160" s="19" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C160" s="8" t="n">
         <v>6.40176960000001</v>
@@ -12691,7 +12699,7 @@
         <v>18</v>
       </c>
       <c r="B161" s="19" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C161" s="8" t="n">
         <v>0</v>
@@ -12758,7 +12766,7 @@
         <v>18</v>
       </c>
       <c r="B162" s="19" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C162" s="8" t="n">
         <v>20.1925496</v>
@@ -12829,7 +12837,7 @@
         <v>18</v>
       </c>
       <c r="B163" s="19" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C163" s="8" t="n">
         <v>23.668175</v>
@@ -12900,24 +12908,24 @@
         <v>18</v>
       </c>
       <c r="B164" s="19" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C164" s="8" t="n">
-        <v>45.2325198</v>
+        <v>49.1075198</v>
       </c>
       <c r="D164" s="8" t="n">
         <v>21</v>
       </c>
       <c r="E164" s="20" t="n">
         <f aca="false">IF(C164&gt;0,D164/C164,"")</f>
-        <v>0.464267745702728</v>
+        <v>0.427633081155933</v>
       </c>
       <c r="F164" s="18" t="str">
         <f aca="false">IF(AND(C164=0,D164&gt;0),"Plant only",IF(AND(D164=0,C164&gt;0),"System only",IF(ABS(D164-C164)&lt;=0.5,"Match",IF(D164&gt;C164,"Plant more","Plant less"))))</f>
         <v>Plant less</v>
       </c>
       <c r="G164" s="8" t="n">
-        <v>45.2325198</v>
+        <v>49.1075198</v>
       </c>
       <c r="H164" s="8" t="n">
         <v>0</v>
@@ -12957,7 +12965,7 @@
         <v>0</v>
       </c>
       <c r="R164" s="21" t="n">
-        <v>22.6793046669932</v>
+        <v>22.7046102499357</v>
       </c>
       <c r="S164" s="22" t="n">
         <v>23</v>
@@ -12971,7 +12979,7 @@
         <v>18</v>
       </c>
       <c r="B165" s="19" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C165" s="8" t="n">
         <v>0</v>
@@ -13038,7 +13046,7 @@
         <v>18</v>
       </c>
       <c r="B166" s="19" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C166" s="8" t="n">
         <v>0</v>
@@ -13103,7 +13111,7 @@
         <v>18</v>
       </c>
       <c r="B167" s="19" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C167" s="8" t="n">
         <v>17.5263252</v>
@@ -13174,7 +13182,7 @@
         <v>18</v>
       </c>
       <c r="B168" s="19" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C168" s="8" t="n">
         <v>45.282544</v>
@@ -13245,7 +13253,7 @@
         <v>18</v>
       </c>
       <c r="B169" s="19" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C169" s="8" t="n">
         <v>3.092136</v>
@@ -13316,7 +13324,7 @@
         <v>18</v>
       </c>
       <c r="B170" s="19" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C170" s="8" t="n">
         <v>0.00544800000000123</v>
@@ -13387,7 +13395,7 @@
         <v>18</v>
       </c>
       <c r="B171" s="19" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C171" s="8" t="n">
         <v>1.46430000000001</v>
@@ -13456,11 +13464,11 @@
     <row r="172" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A172" s="11"/>
       <c r="B172" s="11" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C172" s="12" t="n">
         <f aca="false">SUBTOTAL(9,C5:C171)</f>
-        <v>2520.04662731872</v>
+        <v>2573.49662731872</v>
       </c>
       <c r="D172" s="12" t="n">
         <f aca="false">SUBTOTAL(9,D5:D171)</f>
@@ -13470,15 +13478,15 @@
       <c r="F172" s="11"/>
       <c r="G172" s="12" t="n">
         <f aca="false">SUBTOTAL(9,G5:G171)</f>
-        <v>1961.24320874166</v>
+        <v>2010.72710874166</v>
       </c>
       <c r="H172" s="12" t="n">
         <f aca="false">SUBTOTAL(9,H5:H171)</f>
-        <v>315.272003940105</v>
+        <v>317.198103940105</v>
       </c>
       <c r="I172" s="12" t="n">
         <f aca="false">SUBTOTAL(9,I5:I171)</f>
-        <v>23.2698499498091</v>
+        <v>25.3098499498091</v>
       </c>
       <c r="J172" s="12" t="n">
         <f aca="false">SUBTOTAL(9,J5:J171)</f>
@@ -13486,11 +13494,11 @@
       </c>
       <c r="K172" s="12" t="n">
         <f aca="false">SUBTOTAL(9,K5:K171)</f>
-        <v>1998.76556397618</v>
+        <v>1997.16039909105</v>
       </c>
       <c r="L172" s="12" t="n">
         <f aca="false">SUBTOTAL(9,L5:L171)</f>
-        <v>313.446428005422</v>
+        <v>315.051592890545</v>
       </c>
       <c r="M172" s="12" t="n">
         <f aca="false">SUBTOTAL(9,M5:M171)</f>
@@ -13562,18 +13570,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>2</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>5</v>
@@ -13611,11 +13619,11 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B4" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A4,'Plant x size'!$C$5:$C$171)</f>
-        <v>8.21275760000001</v>
+        <v>12.3127576</v>
       </c>
       <c r="C4" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A4,'Plant x size'!$D$5:$D$171)</f>
@@ -13668,7 +13676,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B5" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A5,'Plant x size'!$C$5:$C$171)</f>
@@ -13725,7 +13733,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B6" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A6,'Plant x size'!$C$5:$C$171)</f>
@@ -13782,7 +13790,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B7" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A7,'Plant x size'!$C$5:$C$171)</f>
@@ -13839,7 +13847,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B8" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A8,'Plant x size'!$C$5:$C$171)</f>
@@ -13896,7 +13904,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B9" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A9,'Plant x size'!$C$5:$C$171)</f>
@@ -13953,7 +13961,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B10" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A10,'Plant x size'!$C$5:$C$171)</f>
@@ -14010,7 +14018,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B11" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A11,'Plant x size'!$C$5:$C$171)</f>
@@ -14067,7 +14075,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B12" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A12,'Plant x size'!$C$5:$C$171)</f>
@@ -14124,7 +14132,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B13" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A13,'Plant x size'!$C$5:$C$171)</f>
@@ -14181,7 +14189,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B14" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A14,'Plant x size'!$C$5:$C$171)</f>
@@ -14238,7 +14246,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="7" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B15" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A15,'Plant x size'!$C$5:$C$171)</f>
@@ -14295,7 +14303,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B16" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A16,'Plant x size'!$C$5:$C$171)</f>
@@ -14352,7 +14360,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="7" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B17" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A17,'Plant x size'!$C$5:$C$171)</f>
@@ -14409,7 +14417,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B18" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A18,'Plant x size'!$C$5:$C$171)</f>
@@ -14466,7 +14474,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="7" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B19" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A19,'Plant x size'!$C$5:$C$171)</f>
@@ -14523,7 +14531,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B20" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A20,'Plant x size'!$C$5:$C$171)</f>
@@ -14580,7 +14588,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="7" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B21" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A21,'Plant x size'!$C$5:$C$171)</f>
@@ -14637,7 +14645,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B22" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A22,'Plant x size'!$C$5:$C$171)</f>
@@ -14694,7 +14702,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B23" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A23,'Plant x size'!$C$5:$C$171)</f>
@@ -14751,11 +14759,11 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B24" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A24,'Plant x size'!$C$5:$C$171)</f>
-        <v>27.9214816</v>
+        <v>33.9614816</v>
       </c>
       <c r="C24" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A24,'Plant x size'!$D$5:$D$171)</f>
@@ -14808,11 +14816,11 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="7" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B25" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A25,'Plant x size'!$C$5:$C$171)</f>
-        <v>18.13226</v>
+        <v>23.10726</v>
       </c>
       <c r="C25" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A25,'Plant x size'!$D$5:$D$171)</f>
@@ -14865,7 +14873,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="7" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B26" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A26,'Plant x size'!$C$5:$C$171)</f>
@@ -14922,7 +14930,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="7" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B27" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A27,'Plant x size'!$C$5:$C$171)</f>
@@ -14979,7 +14987,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="7" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B28" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A28,'Plant x size'!$C$5:$C$171)</f>
@@ -15036,7 +15044,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B29" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A29,'Plant x size'!$C$5:$C$171)</f>
@@ -15093,7 +15101,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B30" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A30,'Plant x size'!$C$5:$C$171)</f>
@@ -15150,7 +15158,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B31" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A31,'Plant x size'!$C$5:$C$171)</f>
@@ -15207,7 +15215,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B32" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A32,'Plant x size'!$C$5:$C$171)</f>
@@ -15264,7 +15272,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B33" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A33,'Plant x size'!$C$5:$C$171)</f>
@@ -15321,7 +15329,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B34" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A34,'Plant x size'!$C$5:$C$171)</f>
@@ -15378,7 +15386,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B35" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A35,'Plant x size'!$C$5:$C$171)</f>
@@ -15435,7 +15443,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B36" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A36,'Plant x size'!$C$5:$C$171)</f>
@@ -15492,11 +15500,11 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B37" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A37,'Plant x size'!$C$5:$C$171)</f>
-        <v>27.7821872</v>
+        <v>30.9021872</v>
       </c>
       <c r="C37" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A37,'Plant x size'!$D$5:$D$171)</f>
@@ -15549,11 +15557,11 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="B38" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A38,'Plant x size'!$C$5:$C$171)</f>
-        <v>4.94651360000001</v>
+        <v>6.94151360000002</v>
       </c>
       <c r="C38" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A38,'Plant x size'!$D$5:$D$171)</f>
@@ -15606,11 +15614,11 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B39" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A39,'Plant x size'!$C$5:$C$171)</f>
-        <v>16.99157</v>
+        <v>22.16657</v>
       </c>
       <c r="C39" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A39,'Plant x size'!$D$5:$D$171)</f>
@@ -15618,11 +15626,11 @@
       </c>
       <c r="D39" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A39,'Plant x size'!$K$5:$K$171)</f>
-        <v>20</v>
+        <v>19.9741088766377</v>
       </c>
       <c r="E39" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A39,'Plant x size'!$L$5:$L$171)</f>
-        <v>8.3</v>
+        <v>8.32589112336227</v>
       </c>
       <c r="F39" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A39,'Plant x size'!$M$5:$M$171)</f>
@@ -15663,7 +15671,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="7" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B40" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A40,'Plant x size'!$C$5:$C$171)</f>
@@ -15720,7 +15728,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="7" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B41" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A41,'Plant x size'!$C$5:$C$171)</f>
@@ -15777,7 +15785,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="7" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B42" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A42,'Plant x size'!$C$5:$C$171)</f>
@@ -15834,7 +15842,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="B43" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A43,'Plant x size'!$C$5:$C$171)</f>
@@ -15891,7 +15899,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="B44" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A44,'Plant x size'!$C$5:$C$171)</f>
@@ -15948,7 +15956,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B45" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A45,'Plant x size'!$C$5:$C$171)</f>
@@ -16005,7 +16013,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B46" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A46,'Plant x size'!$C$5:$C$171)</f>
@@ -16062,7 +16070,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B47" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A47,'Plant x size'!$C$5:$C$171)</f>
@@ -16119,7 +16127,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B48" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A48,'Plant x size'!$C$5:$C$171)</f>
@@ -16176,7 +16184,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B49" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A49,'Plant x size'!$C$5:$C$171)</f>
@@ -16233,7 +16241,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B50" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A50,'Plant x size'!$C$5:$C$171)</f>
@@ -16290,11 +16298,11 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B51" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A51,'Plant x size'!$C$5:$C$171)</f>
-        <v>7.2709284</v>
+        <v>11.3509284</v>
       </c>
       <c r="C51" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A51,'Plant x size'!$D$5:$D$171)</f>
@@ -16347,7 +16355,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B52" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A52,'Plant x size'!$C$5:$C$171)</f>
@@ -16404,7 +16412,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B53" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A53,'Plant x size'!$C$5:$C$171)</f>
@@ -16461,7 +16469,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B54" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A54,'Plant x size'!$C$5:$C$171)</f>
@@ -16518,11 +16526,11 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B55" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A55,'Plant x size'!$C$5:$C$171)</f>
-        <v>59.6501984</v>
+        <v>63.6501984</v>
       </c>
       <c r="C55" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A55,'Plant x size'!$D$5:$D$171)</f>
@@ -16575,7 +16583,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="B56" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A56,'Plant x size'!$C$5:$C$171)</f>
@@ -16632,7 +16640,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B57" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A57,'Plant x size'!$C$5:$C$171)</f>
@@ -16689,7 +16697,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B58" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A58,'Plant x size'!$C$5:$C$171)</f>
@@ -16746,7 +16754,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B59" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A59,'Plant x size'!$C$5:$C$171)</f>
@@ -16803,7 +16811,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B60" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A60,'Plant x size'!$C$5:$C$171)</f>
@@ -16860,7 +16868,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="7" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B61" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A61,'Plant x size'!$C$5:$C$171)</f>
@@ -16917,7 +16925,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="7" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B62" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A62,'Plant x size'!$C$5:$C$171)</f>
@@ -16974,11 +16982,11 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="7" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B63" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A63,'Plant x size'!$C$5:$C$171)</f>
-        <v>146.523296</v>
+        <v>152.523296</v>
       </c>
       <c r="C63" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A63,'Plant x size'!$D$5:$D$171)</f>
@@ -17031,11 +17039,11 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="7" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B64" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A64,'Plant x size'!$C$5:$C$171)</f>
-        <v>100.331245</v>
+        <v>102.231245</v>
       </c>
       <c r="C64" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A64,'Plant x size'!$D$5:$D$171)</f>
@@ -17043,11 +17051,11 @@
       </c>
       <c r="D64" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A64,'Plant x size'!$K$5:$K$171)</f>
-        <v>97.2414805489063</v>
+        <v>95.6622067871455</v>
       </c>
       <c r="E64" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A64,'Plant x size'!$L$5:$L$171)</f>
-        <v>0.642519451093735</v>
+        <v>2.22179321285452</v>
       </c>
       <c r="F64" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A64,'Plant x size'!$M$5:$M$171)</f>
@@ -17088,7 +17096,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="7" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B65" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A65,'Plant x size'!$C$5:$C$171)</f>
@@ -17145,7 +17153,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B66" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A66,'Plant x size'!$C$5:$C$171)</f>
@@ -17202,7 +17210,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="7" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B67" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A67,'Plant x size'!$C$5:$C$171)</f>
@@ -17259,7 +17267,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="7" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B68" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A68,'Plant x size'!$C$5:$C$171)</f>
@@ -17316,7 +17324,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="7" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="B69" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A69,'Plant x size'!$C$5:$C$171)</f>
@@ -17373,7 +17381,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="7" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="B70" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A70,'Plant x size'!$C$5:$C$171)</f>
@@ -17430,7 +17438,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A71" s="7" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B71" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A71,'Plant x size'!$C$5:$C$171)</f>
@@ -17487,7 +17495,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="7" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B72" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A72,'Plant x size'!$C$5:$C$171)</f>
@@ -17544,7 +17552,7 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="7" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B73" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A73,'Plant x size'!$C$5:$C$171)</f>
@@ -17601,7 +17609,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="7" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="B74" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A74,'Plant x size'!$C$5:$C$171)</f>
@@ -17658,11 +17666,11 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A75" s="7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B75" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A75,'Plant x size'!$C$5:$C$171)</f>
-        <v>6.18719324800005</v>
+        <v>12.3371932480001</v>
       </c>
       <c r="C75" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A75,'Plant x size'!$D$5:$D$171)</f>
@@ -17715,7 +17723,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="7" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B76" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A76,'Plant x size'!$C$5:$C$171)</f>
@@ -17772,7 +17780,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="7" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B77" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A77,'Plant x size'!$C$5:$C$171)</f>
@@ -17829,7 +17837,7 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="7" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B78" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A78,'Plant x size'!$C$5:$C$171)</f>
@@ -17886,11 +17894,11 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A79" s="7" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B79" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A79,'Plant x size'!$C$5:$C$171)</f>
-        <v>54.9333268</v>
+        <v>58.8083268</v>
       </c>
       <c r="C79" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A79,'Plant x size'!$D$5:$D$171)</f>
@@ -17943,7 +17951,7 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A80" s="7" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B80" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A80,'Plant x size'!$C$5:$C$171)</f>
@@ -18000,7 +18008,7 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="7" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B81" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A81,'Plant x size'!$C$5:$C$171)</f>
@@ -18057,7 +18065,7 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="7" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B82" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A82,'Plant x size'!$C$5:$C$171)</f>
@@ -18114,7 +18122,7 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="7" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B83" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A83,'Plant x size'!$C$5:$C$171)</f>
@@ -18171,7 +18179,7 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="7" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B84" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A84,'Plant x size'!$C$5:$C$171)</f>
@@ -18228,7 +18236,7 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="7" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B85" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A85,'Plant x size'!$C$5:$C$171)</f>
@@ -18285,7 +18293,7 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="7" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B86" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A86,'Plant x size'!$C$5:$C$171)</f>
@@ -18342,7 +18350,7 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A87" s="7" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B87" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A87,'Plant x size'!$C$5:$C$171)</f>
@@ -18399,7 +18407,7 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A88" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B88" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A88,'Plant x size'!$C$5:$C$171)</f>
@@ -18456,7 +18464,7 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B89" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A89,'Plant x size'!$C$5:$C$171)</f>
@@ -18513,7 +18521,7 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="7" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B90" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A90,'Plant x size'!$C$5:$C$171)</f>
@@ -18570,7 +18578,7 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B91" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A91,'Plant x size'!$C$5:$C$171)</f>
@@ -18627,7 +18635,7 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="7" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B92" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A92,'Plant x size'!$C$5:$C$171)</f>
@@ -18684,7 +18692,7 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A93" s="7" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B93" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A93,'Plant x size'!$C$5:$C$171)</f>
@@ -18741,11 +18749,11 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A94" s="7" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B94" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A94,'Plant x size'!$C$5:$C$171)</f>
-        <v>7.00905037447168</v>
+        <v>9.04905037447167</v>
       </c>
       <c r="C94" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A94,'Plant x size'!$D$5:$D$171)</f>
@@ -18798,7 +18806,7 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A95" s="7" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B95" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A95,'Plant x size'!$C$5:$C$171)</f>
@@ -18855,7 +18863,7 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A96" s="7" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B96" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A96,'Plant x size'!$C$5:$C$171)</f>
@@ -18912,7 +18920,7 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A97" s="7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B97" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A97,'Plant x size'!$C$5:$C$171)</f>
@@ -18969,7 +18977,7 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A98" s="7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B98" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A98,'Plant x size'!$C$5:$C$171)</f>
@@ -19026,7 +19034,7 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A99" s="7" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B99" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A99,'Plant x size'!$C$5:$C$171)</f>
@@ -19083,7 +19091,7 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A100" s="7" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B100" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A100,'Plant x size'!$C$5:$C$171)</f>
@@ -19140,7 +19148,7 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A101" s="7" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B101" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A101,'Plant x size'!$C$5:$C$171)</f>
@@ -19197,7 +19205,7 @@
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A102" s="7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B102" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A102,'Plant x size'!$C$5:$C$171)</f>
@@ -19254,7 +19262,7 @@
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A103" s="7" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B103" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A103,'Plant x size'!$C$5:$C$171)</f>
@@ -19311,7 +19319,7 @@
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A104" s="7" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B104" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A104,'Plant x size'!$C$5:$C$171)</f>
@@ -19368,7 +19376,7 @@
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A105" s="7" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B105" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A105,'Plant x size'!$C$5:$C$171)</f>
@@ -19425,7 +19433,7 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A106" s="7" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B106" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A106,'Plant x size'!$C$5:$C$171)</f>
@@ -19482,7 +19490,7 @@
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A107" s="7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B107" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A107,'Plant x size'!$C$5:$C$171)</f>
@@ -19539,7 +19547,7 @@
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A108" s="7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B108" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A108,'Plant x size'!$C$5:$C$171)</f>
@@ -19596,7 +19604,7 @@
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A109" s="7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B109" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A109,'Plant x size'!$C$5:$C$171)</f>
@@ -19653,7 +19661,7 @@
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A110" s="7" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B110" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A110,'Plant x size'!$C$5:$C$171)</f>
@@ -19710,7 +19718,7 @@
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A111" s="7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B111" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A111,'Plant x size'!$C$5:$C$171)</f>
@@ -19767,7 +19775,7 @@
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A112" s="7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B112" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A112,'Plant x size'!$C$5:$C$171)</f>
@@ -19824,7 +19832,7 @@
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A113" s="7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B113" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A113,'Plant x size'!$C$5:$C$171)</f>
@@ -19881,7 +19889,7 @@
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B114" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A114,'Plant x size'!$C$5:$C$171)</f>
@@ -19938,7 +19946,7 @@
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A115" s="7" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B115" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A115,'Plant x size'!$C$5:$C$171)</f>
@@ -19995,7 +20003,7 @@
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B116" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A116,'Plant x size'!$C$5:$C$171)</f>
@@ -20052,7 +20060,7 @@
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B117" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A117,'Plant x size'!$C$5:$C$171)</f>
@@ -20109,7 +20117,7 @@
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A118" s="7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B118" s="8" t="n">
         <f aca="false">SUMIF('Plant x size'!$B$5:$B$171,A118,'Plant x size'!$C$5:$C$171)</f>
@@ -20166,11 +20174,11 @@
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="11" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B119" s="12" t="n">
         <f aca="false">SUBTOTAL(9,B4:B118)</f>
-        <v>2520.04662731872</v>
+        <v>2573.49662731872</v>
       </c>
       <c r="C119" s="12" t="n">
         <f aca="false">SUBTOTAL(9,C4:C118)</f>
@@ -20178,11 +20186,11 @@
       </c>
       <c r="D119" s="12" t="n">
         <f aca="false">SUBTOTAL(9,D4:D118)</f>
-        <v>1998.76556397618</v>
+        <v>1997.16039909105</v>
       </c>
       <c r="E119" s="12" t="n">
         <f aca="false">SUBTOTAL(9,E4:E118)</f>
-        <v>313.446428005422</v>
+        <v>315.051592890545</v>
       </c>
       <c r="F119" s="12" t="n">
         <f aca="false">SUBTOTAL(9,F4:F118)</f>

</xml_diff>